<commit_message>
Final summary: Cleanup complete, network capture working, auto-detection functional
Co-authored-by: bstHoang <139115555+bstHoang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/batchstudent/1/AnhDThe187386/Results/AnhDThe187386/TC1/GradeDetail.xlsx
+++ b/batchstudent/1/AnhDThe187386/Results/AnhDThe187386/TC1/GradeDetail.xlsx
@@ -1044,7 +1044,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="P2" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="Q2" s="0">
         <x:v>4000</x:v>
@@ -1103,7 +1103,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="Q3" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="R3" s="2" t="s">
         <x:v>47</x:v>
@@ -1156,7 +1156,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="P4" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="Q4" s="0">
         <x:v>4000</x:v>
@@ -1212,7 +1212,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="P5" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="Q5" s="0">
         <x:v>4000</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="Q6" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="R6" s="3" t="s">
         <x:v>55</x:v>
@@ -1327,7 +1327,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="Q7" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
         <x:v>55</x:v>
@@ -1380,7 +1380,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="P8" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="Q8" s="0">
         <x:v>4000</x:v>
@@ -1439,7 +1439,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="Q9" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
         <x:v>55</x:v>
@@ -1492,7 +1492,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="P10" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="Q10" s="0">
         <x:v>4000</x:v>
@@ -1551,7 +1551,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="Q11" s="0">
-        <x:v>46754</x:v>
+        <x:v>58630</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
         <x:v>55</x:v>

</xml_diff>